<commit_message>
adding bedload data points for sand sizes
</commit_message>
<xml_diff>
--- a/data/bedload_tauc/Wilcock2002_tauc.xlsx
+++ b/data/bedload_tauc/Wilcock2002_tauc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\sediment_trap_paper\data\bedload_tauc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3A2038-0735-4234-BFC2-003357074B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F65915-23FC-416C-861F-52415B60469D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3E16E29A-D0FE-4C27-A7A7-0122C151A299}"/>
+    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" activeTab="3" xr2:uid="{3E16E29A-D0FE-4C27-A7A7-0122C151A299}"/>
   </bookViews>
   <sheets>
     <sheet name="Sand GSD calculations" sheetId="4" r:id="rId1"/>
@@ -677,6 +677,9 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -714,9 +717,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -7673,25 +7673,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="J1" s="64" t="s">
+      <c r="J1" s="65" t="s">
         <v>70</v>
       </c>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
     </row>
     <row r="2" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60" t="s">
+      <c r="C2" s="61"/>
+      <c r="D2" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="61"/>
-      <c r="F2" s="62" t="s">
+      <c r="E2" s="62"/>
+      <c r="F2" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="63"/>
+      <c r="G2" s="64"/>
       <c r="J2" s="8" t="s">
         <v>10</v>
       </c>
@@ -7799,8 +7799,8 @@
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="1"/>
-      <c r="P5" s="58"/>
-      <c r="Q5" s="58"/>
+      <c r="P5" s="59"/>
+      <c r="Q5" s="59"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" s="9">
@@ -9407,18 +9407,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="H1" s="67" t="s">
+      <c r="H1" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="65" t="s">
+      <c r="B2" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="66"/>
+      <c r="C2" s="67"/>
       <c r="H2" s="16" t="s">
         <v>14</v>
       </c>
@@ -9785,12 +9785,12 @@
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
-      <c r="H16" s="68" t="s">
+      <c r="H16" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="I16" s="68"/>
-      <c r="J16" s="68"/>
-      <c r="K16" s="68"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="69"/>
+      <c r="K16" s="69"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="22">
@@ -10210,10 +10210,10 @@
       <c r="F1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="69" t="s">
+      <c r="H1" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="69"/>
+      <c r="I1" s="70"/>
       <c r="J1" s="1" t="s">
         <v>0</v>
       </c>
@@ -10242,11 +10242,11 @@
         <f>$I$20+($I$19-$I$20)*EXP(-14*A2)</f>
         <v>1.3290468742698638</v>
       </c>
-      <c r="H2" s="69" t="str">
+      <c r="H2" s="70" t="str">
         <f>B1</f>
         <v>Tri* (Dg/Ds = 10)</v>
       </c>
-      <c r="I2" s="69"/>
+      <c r="I2" s="70"/>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -10374,11 +10374,11 @@
         <f t="shared" si="4"/>
         <v>0.7870350317127095</v>
       </c>
-      <c r="H6" s="69" t="str">
+      <c r="H6" s="70" t="str">
         <f>C1</f>
         <v>Tri* (Dg/Ds = 20)</v>
       </c>
-      <c r="I6" s="69"/>
+      <c r="I6" s="70"/>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -10506,11 +10506,11 @@
         <f t="shared" si="4"/>
         <v>0.4774329545306662</v>
       </c>
-      <c r="H10" s="69" t="str">
+      <c r="H10" s="70" t="str">
         <f>D1</f>
         <v>Tri* (Dg/Ds = 35)</v>
       </c>
-      <c r="I10" s="69"/>
+      <c r="I10" s="70"/>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -10638,11 +10638,11 @@
         <f t="shared" si="4"/>
         <v>0.30058544185786273</v>
       </c>
-      <c r="H14" s="69" t="str">
+      <c r="H14" s="70" t="str">
         <f>E1</f>
         <v>Tri* (Dg/Ds = 50)</v>
       </c>
-      <c r="I14" s="69"/>
+      <c r="I14" s="70"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -10767,11 +10767,11 @@
         <f t="shared" si="4"/>
         <v>0.1995685397000391</v>
       </c>
-      <c r="H18" s="69" t="str">
+      <c r="H18" s="70" t="str">
         <f>F1</f>
         <v>Tri* (Dg/Ds = 43.4)</v>
       </c>
-      <c r="I18" s="69"/>
+      <c r="I18" s="70"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -13049,7 +13049,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE20B856-AC4B-4A0B-8068-FF571A1CD20B}">
-  <dimension ref="A1:M101"/>
+  <dimension ref="A1:M112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" style="1" customWidth="1"/>
@@ -13072,13 +13072,13 @@
       <c r="B1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="70" t="s">
+      <c r="C1" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
       <c r="J1" s="16"/>
@@ -13352,7 +13352,7 @@
       <c r="A17" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B17" s="71">
+      <c r="B17" s="58">
         <f>B7</f>
         <v>0.86746324999999902</v>
       </c>
@@ -13389,7 +13389,7 @@
         <v>45</v>
       </c>
       <c r="B20" s="2">
-        <f t="shared" ref="B20:B29" si="2">$B$7*($B$11-$B$10)*$B$12*($A20/1000000)</f>
+        <f t="shared" ref="B20:B41" si="2">$B$7*($B$11-$B$10)*$B$12*($A20/1000000)</f>
         <v>0.63163795468547745</v>
       </c>
       <c r="C20" s="2"/>
@@ -13410,11 +13410,11 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="B22" s="2">
         <f t="shared" si="2"/>
-        <v>1.403639899301061</v>
+        <v>1.0527299244757955</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -13422,11 +13422,11 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
-        <v>200</v>
+        <v>88</v>
       </c>
       <c r="B23" s="2">
         <f t="shared" si="2"/>
-        <v>2.8072797986021221</v>
+        <v>1.2352031113849335</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -13434,11 +13434,11 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
-        <v>280</v>
+        <v>100</v>
       </c>
       <c r="B24" s="2">
         <f t="shared" si="2"/>
-        <v>3.9301917180429702</v>
+        <v>1.403639899301061</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -13446,11 +13446,11 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
-        <v>500</v>
+        <v>144</v>
       </c>
       <c r="B25" s="2">
         <f t="shared" si="2"/>
-        <v>7.0181994965053045</v>
+        <v>2.0212414549935276</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -13458,11 +13458,11 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="B26" s="2">
         <f t="shared" si="2"/>
-        <v>9.8254792951074261</v>
+        <v>2.8072797986021221</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -13470,11 +13470,11 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
-        <v>850</v>
+        <v>280</v>
       </c>
       <c r="B27" s="2">
         <f t="shared" si="2"/>
-        <v>11.930939144059018</v>
+        <v>3.9301917180429702</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -13482,11 +13482,11 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
-        <v>1000</v>
+        <v>330</v>
       </c>
       <c r="B28" s="2">
         <f t="shared" si="2"/>
-        <v>14.036398993010609</v>
+        <v>4.6320116676935008</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -13494,11 +13494,11 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
-        <v>1500</v>
+        <v>460</v>
       </c>
       <c r="B29" s="2">
         <f t="shared" si="2"/>
-        <v>21.054598489515914</v>
+        <v>6.45674353678488</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -13506,94 +13506,144 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="B30" s="2">
-        <f>$B$7*($B$11-$B$10)*$B$12*($A30/1000000)</f>
-        <v>28.072797986021218</v>
+        <f t="shared" si="2"/>
+        <v>7.0181994965053045</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
+      <c r="A31" s="8">
+        <v>600</v>
+      </c>
+      <c r="B31" s="2">
+        <f t="shared" si="2"/>
+        <v>8.421839395806364</v>
+      </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
-        <v>630</v>
+      <c r="A32" s="8">
+        <v>700</v>
       </c>
       <c r="B32" s="2">
-        <f t="shared" ref="B32" si="3">$B$7*($B$11-$B$10)*$B$12*($A32/1000000)</f>
-        <v>8.8429313655966837</v>
+        <f t="shared" si="2"/>
+        <v>9.8254792951074261</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+      <c r="A33" s="8">
+        <v>850</v>
+      </c>
+      <c r="B33" s="2">
+        <f t="shared" si="2"/>
+        <v>11.930939144059018</v>
+      </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
+      <c r="A34" s="8">
+        <v>900</v>
+      </c>
+      <c r="B34" s="2">
+        <f t="shared" si="2"/>
+        <v>12.632759093709549</v>
+      </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
+      <c r="A35" s="8">
+        <v>1000</v>
+      </c>
+      <c r="B35" s="2">
+        <f t="shared" si="2"/>
+        <v>14.036398993010609</v>
+      </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
+      <c r="A36" s="8">
+        <v>1200</v>
+      </c>
+      <c r="B36" s="2">
+        <f t="shared" si="2"/>
+        <v>16.843678791612728</v>
+      </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
+      <c r="A37" s="8">
+        <v>1400</v>
+      </c>
+      <c r="B37" s="2">
+        <f t="shared" si="2"/>
+        <v>19.650958590214852</v>
+      </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
+      <c r="A38" s="8">
+        <v>1500</v>
+      </c>
+      <c r="B38" s="2">
+        <f t="shared" si="2"/>
+        <v>21.054598489515914</v>
+      </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
+      <c r="A39" s="8">
+        <v>1600</v>
+      </c>
+      <c r="B39" s="2">
+        <f t="shared" si="2"/>
+        <v>22.458238388816977</v>
+      </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
+      <c r="A40" s="8">
+        <v>1800</v>
+      </c>
+      <c r="B40" s="2">
+        <f t="shared" si="2"/>
+        <v>25.265518187419097</v>
+      </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
+      <c r="A41" s="8">
+        <v>2000</v>
+      </c>
+      <c r="B41" s="2">
+        <f t="shared" si="2"/>
+        <v>28.072797986021218</v>
+      </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -13606,8 +13656,13 @@
       <c r="E42" s="2"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
+      <c r="A43" s="2">
+        <v>630</v>
+      </c>
+      <c r="B43" s="2">
+        <f t="shared" ref="B43" si="3">$B$7*($B$11-$B$10)*$B$12*($A43/1000000)</f>
+        <v>8.8429313655966837</v>
+      </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -14017,6 +14072,83 @@
       <c r="C101" s="2"/>
       <c r="D101" s="2"/>
       <c r="E101" s="2"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="2"/>
+      <c r="B102" s="2"/>
+      <c r="C102" s="2"/>
+      <c r="D102" s="2"/>
+      <c r="E102" s="2"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" s="2"/>
+      <c r="B103" s="2"/>
+      <c r="C103" s="2"/>
+      <c r="D103" s="2"/>
+      <c r="E103" s="2"/>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" s="2"/>
+      <c r="B104" s="2"/>
+      <c r="C104" s="2"/>
+      <c r="D104" s="2"/>
+      <c r="E104" s="2"/>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" s="2"/>
+      <c r="B105" s="2"/>
+      <c r="C105" s="2"/>
+      <c r="D105" s="2"/>
+      <c r="E105" s="2"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" s="2"/>
+      <c r="B106" s="2"/>
+      <c r="C106" s="2"/>
+      <c r="D106" s="2"/>
+      <c r="E106" s="2"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" s="2"/>
+      <c r="B107" s="2"/>
+      <c r="C107" s="2"/>
+      <c r="D107" s="2"/>
+      <c r="E107" s="2"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" s="2"/>
+      <c r="B108" s="2"/>
+      <c r="C108" s="2"/>
+      <c r="D108" s="2"/>
+      <c r="E108" s="2"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="2"/>
+      <c r="B109" s="2"/>
+      <c r="C109" s="2"/>
+      <c r="D109" s="2"/>
+      <c r="E109" s="2"/>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="2"/>
+      <c r="B110" s="2"/>
+      <c r="C110" s="2"/>
+      <c r="D110" s="2"/>
+      <c r="E110" s="2"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="2"/>
+      <c r="B111" s="2"/>
+      <c r="C111" s="2"/>
+      <c r="D111" s="2"/>
+      <c r="E111" s="2"/>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" s="2"/>
+      <c r="B112" s="2"/>
+      <c r="C112" s="2"/>
+      <c r="D112" s="2"/>
+      <c r="E112" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
updating u*/ws plots and VHF periods for final version
</commit_message>
<xml_diff>
--- a/data/bedload_tauc/Wilcock2002_tauc.xlsx
+++ b/data/bedload_tauc/Wilcock2002_tauc.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\sediment_trap_paper\data\bedload_tauc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F65915-23FC-416C-861F-52415B60469D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E04FD6-7613-407A-8EB7-F2C8320888B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" activeTab="3" xr2:uid="{3E16E29A-D0FE-4C27-A7A7-0122C151A299}"/>
   </bookViews>
@@ -680,6 +680,9 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -714,9 +717,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -7673,25 +7673,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="J1" s="65" t="s">
+      <c r="J1" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
     </row>
     <row r="2" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61" t="s">
+      <c r="C2" s="62"/>
+      <c r="D2" s="62" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="62"/>
-      <c r="F2" s="63" t="s">
+      <c r="E2" s="63"/>
+      <c r="F2" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="64"/>
+      <c r="G2" s="65"/>
       <c r="J2" s="8" t="s">
         <v>10</v>
       </c>
@@ -7799,8 +7799,8 @@
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="1"/>
-      <c r="P5" s="59"/>
-      <c r="Q5" s="59"/>
+      <c r="P5" s="60"/>
+      <c r="Q5" s="60"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" s="9">
@@ -9407,18 +9407,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="H1" s="68" t="s">
+      <c r="H1" s="69" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="67"/>
+      <c r="C2" s="68"/>
       <c r="H2" s="16" t="s">
         <v>14</v>
       </c>
@@ -9785,12 +9785,12 @@
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
-      <c r="H16" s="69" t="s">
+      <c r="H16" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="I16" s="69"/>
-      <c r="J16" s="69"/>
-      <c r="K16" s="69"/>
+      <c r="I16" s="70"/>
+      <c r="J16" s="70"/>
+      <c r="K16" s="70"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="22">
@@ -10210,10 +10210,10 @@
       <c r="F1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="70" t="s">
+      <c r="H1" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="70"/>
+      <c r="I1" s="71"/>
       <c r="J1" s="1" t="s">
         <v>0</v>
       </c>
@@ -10242,11 +10242,11 @@
         <f>$I$20+($I$19-$I$20)*EXP(-14*A2)</f>
         <v>1.3290468742698638</v>
       </c>
-      <c r="H2" s="70" t="str">
+      <c r="H2" s="71" t="str">
         <f>B1</f>
         <v>Tri* (Dg/Ds = 10)</v>
       </c>
-      <c r="I2" s="70"/>
+      <c r="I2" s="71"/>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -10374,11 +10374,11 @@
         <f t="shared" si="4"/>
         <v>0.7870350317127095</v>
       </c>
-      <c r="H6" s="70" t="str">
+      <c r="H6" s="71" t="str">
         <f>C1</f>
         <v>Tri* (Dg/Ds = 20)</v>
       </c>
-      <c r="I6" s="70"/>
+      <c r="I6" s="71"/>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -10506,11 +10506,11 @@
         <f t="shared" si="4"/>
         <v>0.4774329545306662</v>
       </c>
-      <c r="H10" s="70" t="str">
+      <c r="H10" s="71" t="str">
         <f>D1</f>
         <v>Tri* (Dg/Ds = 35)</v>
       </c>
-      <c r="I10" s="70"/>
+      <c r="I10" s="71"/>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -10638,11 +10638,11 @@
         <f t="shared" si="4"/>
         <v>0.30058544185786273</v>
       </c>
-      <c r="H14" s="70" t="str">
+      <c r="H14" s="71" t="str">
         <f>E1</f>
         <v>Tri* (Dg/Ds = 50)</v>
       </c>
-      <c r="I14" s="70"/>
+      <c r="I14" s="71"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -10767,11 +10767,11 @@
         <f t="shared" si="4"/>
         <v>0.1995685397000391</v>
       </c>
-      <c r="H18" s="70" t="str">
+      <c r="H18" s="71" t="str">
         <f>F1</f>
         <v>Tri* (Dg/Ds = 43.4)</v>
       </c>
-      <c r="I18" s="70"/>
+      <c r="I18" s="71"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -13049,7 +13049,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE20B856-AC4B-4A0B-8068-FF571A1CD20B}">
-  <dimension ref="A1:M112"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" style="1" customWidth="1"/>
@@ -13072,13 +13072,13 @@
       <c r="B1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="71" t="s">
+      <c r="C1" s="59" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
       <c r="J1" s="16"/>
@@ -13389,7 +13389,7 @@
         <v>45</v>
       </c>
       <c r="B20" s="2">
-        <f t="shared" ref="B20:B41" si="2">$B$7*($B$11-$B$10)*$B$12*($A20/1000000)</f>
+        <f t="shared" ref="B20:B44" si="2">$B$7*($B$11-$B$10)*$B$12*($A20/1000000)</f>
         <v>0.63163795468547745</v>
       </c>
       <c r="C20" s="2"/>
@@ -13518,11 +13518,11 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="B31" s="2">
         <f t="shared" si="2"/>
-        <v>8.421839395806364</v>
+        <v>7.7200194461558356</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -13530,11 +13530,11 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="B32" s="2">
         <f t="shared" si="2"/>
-        <v>9.8254792951074261</v>
+        <v>8.421839395806364</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -13542,11 +13542,11 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
-        <v>850</v>
+        <v>650</v>
       </c>
       <c r="B33" s="2">
         <f t="shared" si="2"/>
-        <v>11.930939144059018</v>
+        <v>9.1236593454568951</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -13554,11 +13554,11 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="8">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="B34" s="2">
         <f t="shared" si="2"/>
-        <v>12.632759093709549</v>
+        <v>9.8254792951074261</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -13566,11 +13566,11 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="8">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="B35" s="2">
         <f t="shared" si="2"/>
-        <v>14.036398993010609</v>
+        <v>10.527299244757957</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -13578,11 +13578,11 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="8">
-        <v>1200</v>
+        <v>850</v>
       </c>
       <c r="B36" s="2">
         <f t="shared" si="2"/>
-        <v>16.843678791612728</v>
+        <v>11.930939144059018</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -13590,11 +13590,11 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="8">
-        <v>1400</v>
+        <v>900</v>
       </c>
       <c r="B37" s="2">
         <f t="shared" si="2"/>
-        <v>19.650958590214852</v>
+        <v>12.632759093709549</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -13602,11 +13602,11 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="B38" s="2">
         <f t="shared" si="2"/>
-        <v>21.054598489515914</v>
+        <v>14.036398993010609</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -13614,11 +13614,11 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="B39" s="2">
         <f t="shared" si="2"/>
-        <v>22.458238388816977</v>
+        <v>16.843678791612728</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -13626,11 +13626,11 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
-        <v>1800</v>
+        <v>1400</v>
       </c>
       <c r="B40" s="2">
         <f t="shared" si="2"/>
-        <v>25.265518187419097</v>
+        <v>19.650958590214852</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -13638,38 +13638,48 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="B41" s="2">
         <f t="shared" si="2"/>
-        <v>28.072797986021218</v>
+        <v>21.054598489515914</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
+      <c r="A42" s="8">
+        <v>1600</v>
+      </c>
+      <c r="B42" s="2">
+        <f t="shared" si="2"/>
+        <v>22.458238388816977</v>
+      </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
-        <v>630</v>
+      <c r="A43" s="8">
+        <v>1800</v>
       </c>
       <c r="B43" s="2">
-        <f t="shared" ref="B43" si="3">$B$7*($B$11-$B$10)*$B$12*($A43/1000000)</f>
-        <v>8.8429313655966837</v>
+        <f t="shared" si="2"/>
+        <v>25.265518187419097</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
+      <c r="A44" s="8">
+        <v>2000</v>
+      </c>
+      <c r="B44" s="2">
+        <f t="shared" si="2"/>
+        <v>28.072797986021218</v>
+      </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -13682,8 +13692,13 @@
       <c r="E45" s="2"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
+      <c r="A46" s="2">
+        <v>630</v>
+      </c>
+      <c r="B46" s="2">
+        <f t="shared" ref="B46" si="3">$B$7*($B$11-$B$10)*$B$12*($A46/1000000)</f>
+        <v>8.8429313655966837</v>
+      </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
@@ -14149,6 +14164,27 @@
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
       <c r="E112" s="2"/>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="2"/>
+      <c r="B113" s="2"/>
+      <c r="C113" s="2"/>
+      <c r="D113" s="2"/>
+      <c r="E113" s="2"/>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="2"/>
+      <c r="B114" s="2"/>
+      <c r="C114" s="2"/>
+      <c r="D114" s="2"/>
+      <c r="E114" s="2"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="2"/>
+      <c r="B115" s="2"/>
+      <c r="C115" s="2"/>
+      <c r="D115" s="2"/>
+      <c r="E115" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
calculating d16 of the bed
</commit_message>
<xml_diff>
--- a/data/bedload_tauc/Wilcock2002_tauc.xlsx
+++ b/data/bedload_tauc/Wilcock2002_tauc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\sediment_trap_paper\data\bedload_tauc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E04FD6-7613-407A-8EB7-F2C8320888B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9A810B-0CE2-48C2-BF3F-A01A8FA2E068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" activeTab="3" xr2:uid="{3E16E29A-D0FE-4C27-A7A7-0122C151A299}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E16E29A-D0FE-4C27-A7A7-0122C151A299}"/>
   </bookViews>
   <sheets>
     <sheet name="Sand GSD calculations" sheetId="4" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
   <si>
     <t>Fs</t>
   </si>
@@ -285,6 +285,15 @@
   </si>
   <si>
     <t xml:space="preserve">using Tri* = </t>
+  </si>
+  <si>
+    <t>Bed D50</t>
+  </si>
+  <si>
+    <t>Bed D84</t>
+  </si>
+  <si>
+    <t>Bed D16</t>
   </si>
 </sst>
 </file>
@@ -7798,7 +7807,9 @@
         <v>1.9242283205873113E-2</v>
       </c>
       <c r="M5" s="2"/>
-      <c r="N5" s="1"/>
+      <c r="N5" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="P5" s="60"/>
       <c r="Q5" s="60"/>
     </row>
@@ -7837,7 +7848,12 @@
         <v>1.990567778890236E-2</v>
       </c>
       <c r="M6" s="2"/>
-      <c r="N6" s="1"/>
+      <c r="N6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="P6" s="16"/>
       <c r="Q6" s="16"/>
       <c r="R6" s="16"/>
@@ -7878,7 +7894,14 @@
         <v>4.5248868831398781E-2</v>
       </c>
       <c r="M7" s="2"/>
-      <c r="N7" s="1"/>
+      <c r="N7" s="14">
+        <f>E12</f>
+        <v>31.753554502369667</v>
+      </c>
+      <c r="O7" s="11">
+        <f>B12</f>
+        <v>32</v>
+      </c>
       <c r="P7" s="1"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
@@ -7919,7 +7942,13 @@
         <v>4.6153846206964395E-2</v>
       </c>
       <c r="M8" s="2"/>
-      <c r="N8" s="1"/>
+      <c r="N8" s="18">
+        <v>50</v>
+      </c>
+      <c r="O8" s="19">
+        <f>O7 + (N8 - N7) * ((O9 - O7) / (N9 - N7))</f>
+        <v>43.639534883720927</v>
+      </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
@@ -7960,7 +7989,14 @@
         <v>4.7511312270312807E-2</v>
       </c>
       <c r="M9" s="2"/>
-      <c r="N9" s="1"/>
+      <c r="N9" s="14">
+        <f>E13</f>
+        <v>52.132701421800952</v>
+      </c>
+      <c r="O9" s="11">
+        <f>B13</f>
+        <v>45</v>
+      </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="2"/>
       <c r="R9" s="2"/>
@@ -8083,7 +8119,9 @@
         <v>5.565610865040331E-2</v>
       </c>
       <c r="M12" s="2"/>
-      <c r="N12" s="1"/>
+      <c r="N12" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="2"/>
       <c r="R12" s="2"/>
@@ -8124,7 +8162,12 @@
         <v>6.108597290379697E-2</v>
       </c>
       <c r="M13" s="2"/>
-      <c r="N13" s="1"/>
+      <c r="N13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="P13" s="1"/>
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
@@ -8165,7 +8208,14 @@
         <v>6.7873303220539055E-2</v>
       </c>
       <c r="M14" s="2"/>
-      <c r="N14" s="1"/>
+      <c r="N14" s="14">
+        <f>E14</f>
+        <v>72.511848341232238</v>
+      </c>
+      <c r="O14" s="11">
+        <f>B14</f>
+        <v>64</v>
+      </c>
       <c r="P14" s="1"/>
       <c r="Q14" s="2"/>
       <c r="R14" s="2"/>
@@ -8206,7 +8256,13 @@
         <v>0.1131221719988196</v>
       </c>
       <c r="M15" s="2"/>
-      <c r="N15" s="1"/>
+      <c r="N15" s="18">
+        <v>84</v>
+      </c>
+      <c r="O15" s="19">
+        <f>O14 + (N15 - N14) * ((O16 - O14) / (N16 - N14))</f>
+        <v>82.006857142857143</v>
+      </c>
       <c r="P15" s="1"/>
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
@@ -8247,7 +8303,14 @@
         <v>0.22624434394452098</v>
       </c>
       <c r="M16" s="2"/>
-      <c r="N16" s="1"/>
+      <c r="N16" s="14">
+        <f>E15</f>
+        <v>89.099526066350705</v>
+      </c>
+      <c r="O16" s="11">
+        <f>B15</f>
+        <v>90</v>
+      </c>
       <c r="P16" s="1"/>
       <c r="Q16" s="2"/>
       <c r="R16" s="2"/>
@@ -8352,7 +8415,9 @@
         <v>0.73755656113909107</v>
       </c>
       <c r="M19" s="2"/>
-      <c r="N19" s="1"/>
+      <c r="N19" s="1" t="s">
+        <v>75</v>
+      </c>
       <c r="P19" s="1"/>
       <c r="Q19" s="2"/>
       <c r="R19" s="2"/>
@@ -8382,7 +8447,12 @@
         <v>0.89592760186307296</v>
       </c>
       <c r="M20" s="2"/>
-      <c r="N20" s="1"/>
+      <c r="N20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="P20" s="1"/>
       <c r="Q20" s="2"/>
       <c r="R20" s="2"/>
@@ -8408,7 +8478,14 @@
         <v>0.94117647064135346</v>
       </c>
       <c r="M21" s="2"/>
-      <c r="N21" s="1"/>
+      <c r="N21" s="14">
+        <f>E10</f>
+        <v>7.109004739336493</v>
+      </c>
+      <c r="O21" s="11">
+        <f>B10</f>
+        <v>16</v>
+      </c>
       <c r="P21" s="1"/>
       <c r="Q21" s="2"/>
       <c r="R21" s="2"/>
@@ -8437,7 +8514,13 @@
         <v>1.0000000000531182</v>
       </c>
       <c r="M22" s="2"/>
-      <c r="N22" s="1"/>
+      <c r="N22" s="18">
+        <v>16</v>
+      </c>
+      <c r="O22" s="19">
+        <f>O21 + (N22 - N21) * ((O23 - O21) / (N23 - N21))</f>
+        <v>20.952640000000002</v>
+      </c>
       <c r="P22" s="1"/>
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
@@ -8456,7 +8539,14 @@
       <c r="J23" s="9"/>
       <c r="K23" s="10"/>
       <c r="L23" s="10"/>
-      <c r="N23" s="1"/>
+      <c r="N23" s="14">
+        <f>E11</f>
+        <v>18.957345971563981</v>
+      </c>
+      <c r="O23" s="11">
+        <f>B11</f>
+        <v>22.6</v>
+      </c>
       <c r="P23" s="1"/>
       <c r="Q23" s="2"/>
       <c r="R23" s="2"/>

</xml_diff>

<commit_message>
additional checks for reviewer comments (1)
</commit_message>
<xml_diff>
--- a/data/bedload_tauc/Wilcock2002_tauc.xlsx
+++ b/data/bedload_tauc/Wilcock2002_tauc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\sediment_trap_paper\data\bedload_tauc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9A810B-0CE2-48C2-BF3F-A01A8FA2E068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A266EC8-11B7-4750-A04D-EED28B7EBD23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E16E29A-D0FE-4C27-A7A7-0122C151A299}"/>
   </bookViews>
@@ -689,9 +689,6 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -726,6 +723,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -7682,25 +7682,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="J1" s="66" t="s">
+      <c r="J1" s="65" t="s">
         <v>70</v>
       </c>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
     </row>
     <row r="2" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62" t="s">
+      <c r="C2" s="61"/>
+      <c r="D2" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="63"/>
-      <c r="F2" s="64" t="s">
+      <c r="E2" s="62"/>
+      <c r="F2" s="63" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="65"/>
+      <c r="G2" s="64"/>
       <c r="J2" s="8" t="s">
         <v>10</v>
       </c>
@@ -7810,8 +7810,8 @@
       <c r="N5" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="P5" s="60"/>
-      <c r="Q5" s="60"/>
+      <c r="P5" s="59"/>
+      <c r="Q5" s="59"/>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" s="9">
@@ -9497,18 +9497,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="H1" s="69" t="s">
+      <c r="H1" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="67" t="s">
+      <c r="B2" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="68"/>
+      <c r="C2" s="67"/>
       <c r="H2" s="16" t="s">
         <v>14</v>
       </c>
@@ -9875,12 +9875,12 @@
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
-      <c r="H16" s="70" t="s">
+      <c r="H16" s="69" t="s">
         <v>21</v>
       </c>
-      <c r="I16" s="70"/>
-      <c r="J16" s="70"/>
-      <c r="K16" s="70"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="69"/>
+      <c r="K16" s="69"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="22">
@@ -10300,10 +10300,10 @@
       <c r="F1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="71" t="s">
+      <c r="H1" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="71"/>
+      <c r="I1" s="70"/>
       <c r="J1" s="1" t="s">
         <v>0</v>
       </c>
@@ -10332,11 +10332,11 @@
         <f>$I$20+($I$19-$I$20)*EXP(-14*A2)</f>
         <v>1.3290468742698638</v>
       </c>
-      <c r="H2" s="71" t="str">
+      <c r="H2" s="70" t="str">
         <f>B1</f>
         <v>Tri* (Dg/Ds = 10)</v>
       </c>
-      <c r="I2" s="71"/>
+      <c r="I2" s="70"/>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -10464,11 +10464,11 @@
         <f t="shared" si="4"/>
         <v>0.7870350317127095</v>
       </c>
-      <c r="H6" s="71" t="str">
+      <c r="H6" s="70" t="str">
         <f>C1</f>
         <v>Tri* (Dg/Ds = 20)</v>
       </c>
-      <c r="I6" s="71"/>
+      <c r="I6" s="70"/>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -10596,11 +10596,11 @@
         <f t="shared" si="4"/>
         <v>0.4774329545306662</v>
       </c>
-      <c r="H10" s="71" t="str">
+      <c r="H10" s="70" t="str">
         <f>D1</f>
         <v>Tri* (Dg/Ds = 35)</v>
       </c>
-      <c r="I10" s="71"/>
+      <c r="I10" s="70"/>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -10728,11 +10728,11 @@
         <f t="shared" si="4"/>
         <v>0.30058544185786273</v>
       </c>
-      <c r="H14" s="71" t="str">
+      <c r="H14" s="70" t="str">
         <f>E1</f>
         <v>Tri* (Dg/Ds = 50)</v>
       </c>
-      <c r="I14" s="71"/>
+      <c r="I14" s="70"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -10857,11 +10857,11 @@
         <f t="shared" si="4"/>
         <v>0.1995685397000391</v>
       </c>
-      <c r="H18" s="71" t="str">
+      <c r="H18" s="70" t="str">
         <f>F1</f>
         <v>Tri* (Dg/Ds = 43.4)</v>
       </c>
-      <c r="I18" s="71"/>
+      <c r="I18" s="70"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -13162,13 +13162,13 @@
       <c r="B1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="71" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
       <c r="J1" s="16"/>

</xml_diff>